<commit_message>
Full pipeline validated: n=95 patients, empty lines eliminated and score top-5 verified.
</commit_message>
<xml_diff>
--- a/data/processed/Matrice_Complete_IMA_Clean.xlsx
+++ b/data/processed/Matrice_Complete_IMA_Clean.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:MZ97"/>
+  <dimension ref="A1:MZ96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -97408,392 +97408,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" t="inlineStr"/>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
-      <c r="M97" t="inlineStr"/>
-      <c r="N97" t="inlineStr"/>
-      <c r="O97" t="inlineStr"/>
-      <c r="P97" t="inlineStr"/>
-      <c r="Q97" t="inlineStr"/>
-      <c r="R97" t="inlineStr"/>
-      <c r="S97" t="inlineStr"/>
-      <c r="T97" t="inlineStr"/>
-      <c r="U97" t="inlineStr"/>
-      <c r="V97" t="inlineStr"/>
-      <c r="W97" t="inlineStr"/>
-      <c r="X97" t="inlineStr"/>
-      <c r="Y97" t="inlineStr"/>
-      <c r="Z97" t="inlineStr"/>
-      <c r="AA97" t="inlineStr"/>
-      <c r="AB97" t="inlineStr"/>
-      <c r="AC97" t="inlineStr"/>
-      <c r="AD97" t="inlineStr"/>
-      <c r="AE97" t="inlineStr"/>
-      <c r="AF97" t="inlineStr"/>
-      <c r="AG97" t="inlineStr"/>
-      <c r="AH97" t="inlineStr"/>
-      <c r="AI97" t="inlineStr"/>
-      <c r="AJ97" t="inlineStr"/>
-      <c r="AK97" t="inlineStr"/>
-      <c r="AL97" t="inlineStr"/>
-      <c r="AM97" t="inlineStr"/>
-      <c r="AN97" t="inlineStr"/>
-      <c r="AO97" t="inlineStr"/>
-      <c r="AP97" t="inlineStr"/>
-      <c r="AQ97" t="inlineStr"/>
-      <c r="AR97" t="inlineStr"/>
-      <c r="AS97" t="inlineStr"/>
-      <c r="AT97" t="inlineStr"/>
-      <c r="AU97" t="inlineStr"/>
-      <c r="AV97" t="inlineStr"/>
-      <c r="AW97" t="inlineStr"/>
-      <c r="AX97" t="inlineStr"/>
-      <c r="AY97" t="inlineStr"/>
-      <c r="AZ97" t="inlineStr"/>
-      <c r="BA97" t="inlineStr"/>
-      <c r="BB97" t="inlineStr"/>
-      <c r="BC97" t="inlineStr"/>
-      <c r="BD97" t="inlineStr"/>
-      <c r="BE97" t="inlineStr"/>
-      <c r="BF97" t="inlineStr"/>
-      <c r="BG97" t="inlineStr"/>
-      <c r="BH97" t="inlineStr"/>
-      <c r="BI97" t="inlineStr"/>
-      <c r="BJ97" t="inlineStr"/>
-      <c r="BK97" t="inlineStr"/>
-      <c r="BL97" t="inlineStr"/>
-      <c r="BM97" t="inlineStr"/>
-      <c r="BN97" t="inlineStr"/>
-      <c r="BO97" t="inlineStr"/>
-      <c r="BP97" t="inlineStr"/>
-      <c r="BQ97" t="inlineStr"/>
-      <c r="BR97" t="inlineStr"/>
-      <c r="BS97" t="inlineStr"/>
-      <c r="BT97" t="inlineStr"/>
-      <c r="BU97" t="inlineStr"/>
-      <c r="BV97" t="inlineStr"/>
-      <c r="BW97" t="inlineStr"/>
-      <c r="BX97" t="inlineStr"/>
-      <c r="BY97" t="inlineStr"/>
-      <c r="BZ97" t="inlineStr"/>
-      <c r="CA97" t="inlineStr"/>
-      <c r="CB97" t="inlineStr"/>
-      <c r="CC97" t="inlineStr"/>
-      <c r="CD97" t="inlineStr"/>
-      <c r="CE97" t="n">
-        <v>6</v>
-      </c>
-      <c r="CF97" t="n">
-        <v>8</v>
-      </c>
-      <c r="CG97" t="n">
-        <v>3</v>
-      </c>
-      <c r="CH97" t="n">
-        <v>15</v>
-      </c>
-      <c r="CI97" t="n">
-        <v>7</v>
-      </c>
-      <c r="CJ97" t="n">
-        <v>9</v>
-      </c>
-      <c r="CK97" t="n">
-        <v>0</v>
-      </c>
-      <c r="CL97" t="n">
-        <v>9</v>
-      </c>
-      <c r="CM97" t="n">
-        <v>4</v>
-      </c>
-      <c r="CN97" t="n">
-        <v>2</v>
-      </c>
-      <c r="CO97" t="inlineStr"/>
-      <c r="CP97" t="inlineStr"/>
-      <c r="CQ97" t="inlineStr"/>
-      <c r="CR97" t="inlineStr"/>
-      <c r="CS97" t="inlineStr"/>
-      <c r="CT97" t="inlineStr"/>
-      <c r="CU97" t="inlineStr"/>
-      <c r="CV97" t="inlineStr"/>
-      <c r="CW97" t="inlineStr"/>
-      <c r="CX97" t="inlineStr"/>
-      <c r="CY97" t="inlineStr"/>
-      <c r="CZ97" t="inlineStr"/>
-      <c r="DA97" t="inlineStr"/>
-      <c r="DB97" t="inlineStr"/>
-      <c r="DC97" t="inlineStr"/>
-      <c r="DD97" t="inlineStr"/>
-      <c r="DE97" t="inlineStr"/>
-      <c r="DF97" t="inlineStr"/>
-      <c r="DG97" t="inlineStr"/>
-      <c r="DH97" t="inlineStr"/>
-      <c r="DI97" t="inlineStr"/>
-      <c r="DJ97" t="inlineStr"/>
-      <c r="DK97" t="inlineStr"/>
-      <c r="DL97" t="inlineStr"/>
-      <c r="DM97" t="inlineStr"/>
-      <c r="DN97" t="inlineStr"/>
-      <c r="DO97" t="inlineStr"/>
-      <c r="DP97" t="inlineStr"/>
-      <c r="DQ97" t="inlineStr"/>
-      <c r="DR97" t="inlineStr"/>
-      <c r="DS97" t="inlineStr"/>
-      <c r="DT97" t="inlineStr"/>
-      <c r="DU97" t="inlineStr"/>
-      <c r="DV97" t="inlineStr"/>
-      <c r="DW97" t="inlineStr"/>
-      <c r="DX97" t="inlineStr"/>
-      <c r="DY97" t="inlineStr"/>
-      <c r="DZ97" t="inlineStr"/>
-      <c r="EA97" t="inlineStr"/>
-      <c r="EB97" t="inlineStr"/>
-      <c r="EC97" t="inlineStr"/>
-      <c r="ED97" t="inlineStr"/>
-      <c r="EE97" t="inlineStr"/>
-      <c r="EF97" t="inlineStr"/>
-      <c r="EG97" t="inlineStr"/>
-      <c r="EH97" t="inlineStr"/>
-      <c r="EI97" t="inlineStr"/>
-      <c r="EJ97" t="inlineStr"/>
-      <c r="EK97" t="inlineStr"/>
-      <c r="EL97" t="inlineStr"/>
-      <c r="EM97" t="inlineStr"/>
-      <c r="EN97" t="inlineStr"/>
-      <c r="EO97" t="inlineStr"/>
-      <c r="EP97" t="inlineStr"/>
-      <c r="EQ97" t="inlineStr"/>
-      <c r="ER97" t="inlineStr"/>
-      <c r="ES97" t="inlineStr"/>
-      <c r="ET97" t="inlineStr"/>
-      <c r="EU97" t="inlineStr"/>
-      <c r="EV97" t="inlineStr"/>
-      <c r="EW97" t="inlineStr"/>
-      <c r="EX97" t="inlineStr"/>
-      <c r="EY97" t="inlineStr"/>
-      <c r="EZ97" t="inlineStr"/>
-      <c r="FA97" t="inlineStr"/>
-      <c r="FB97" t="inlineStr"/>
-      <c r="FC97" t="inlineStr"/>
-      <c r="FD97" t="inlineStr"/>
-      <c r="FE97" t="inlineStr"/>
-      <c r="FF97" t="inlineStr"/>
-      <c r="FG97" t="inlineStr"/>
-      <c r="FH97" t="inlineStr"/>
-      <c r="FI97" t="inlineStr"/>
-      <c r="FJ97" t="inlineStr"/>
-      <c r="FK97" t="inlineStr"/>
-      <c r="FL97" t="inlineStr"/>
-      <c r="FM97" t="inlineStr"/>
-      <c r="FN97" t="inlineStr"/>
-      <c r="FO97" t="inlineStr"/>
-      <c r="FP97" t="inlineStr"/>
-      <c r="FQ97" t="inlineStr"/>
-      <c r="FR97" t="inlineStr"/>
-      <c r="FS97" t="inlineStr"/>
-      <c r="FT97" t="inlineStr"/>
-      <c r="FU97" t="inlineStr"/>
-      <c r="FV97" t="inlineStr"/>
-      <c r="FW97" t="inlineStr"/>
-      <c r="FX97" t="inlineStr"/>
-      <c r="FY97" t="inlineStr"/>
-      <c r="FZ97" t="inlineStr"/>
-      <c r="GA97" t="inlineStr"/>
-      <c r="GB97" t="inlineStr"/>
-      <c r="GC97" t="inlineStr"/>
-      <c r="GD97" t="inlineStr"/>
-      <c r="GE97" t="inlineStr"/>
-      <c r="GF97" t="inlineStr"/>
-      <c r="GG97" t="inlineStr"/>
-      <c r="GH97" t="inlineStr"/>
-      <c r="GI97" t="inlineStr"/>
-      <c r="GJ97" t="inlineStr"/>
-      <c r="GK97" t="inlineStr"/>
-      <c r="GL97" t="inlineStr"/>
-      <c r="GM97" t="inlineStr"/>
-      <c r="GN97" t="inlineStr"/>
-      <c r="GO97" t="inlineStr"/>
-      <c r="GP97" t="inlineStr"/>
-      <c r="GQ97" t="inlineStr"/>
-      <c r="GR97" t="inlineStr"/>
-      <c r="GS97" t="inlineStr"/>
-      <c r="GT97" t="inlineStr"/>
-      <c r="GU97" t="inlineStr"/>
-      <c r="GV97" t="inlineStr"/>
-      <c r="GW97" t="inlineStr"/>
-      <c r="GX97" t="inlineStr"/>
-      <c r="GY97" t="inlineStr"/>
-      <c r="GZ97" t="inlineStr"/>
-      <c r="HA97" t="inlineStr"/>
-      <c r="HB97" t="inlineStr"/>
-      <c r="HC97" t="inlineStr"/>
-      <c r="HD97" t="inlineStr"/>
-      <c r="HE97" t="inlineStr"/>
-      <c r="HF97" t="inlineStr"/>
-      <c r="HG97" t="inlineStr"/>
-      <c r="HH97" t="inlineStr"/>
-      <c r="HI97" t="inlineStr"/>
-      <c r="HJ97" t="inlineStr"/>
-      <c r="HK97" t="inlineStr"/>
-      <c r="HL97" t="inlineStr"/>
-      <c r="HM97" t="inlineStr"/>
-      <c r="HN97" t="inlineStr"/>
-      <c r="HO97" t="inlineStr"/>
-      <c r="HP97" t="inlineStr"/>
-      <c r="HQ97" t="inlineStr"/>
-      <c r="HR97" t="inlineStr"/>
-      <c r="HS97" t="inlineStr"/>
-      <c r="HT97" t="inlineStr"/>
-      <c r="HU97" t="inlineStr"/>
-      <c r="HV97" t="inlineStr"/>
-      <c r="HW97" t="inlineStr"/>
-      <c r="HX97" t="inlineStr"/>
-      <c r="HY97" t="inlineStr"/>
-      <c r="HZ97" t="inlineStr"/>
-      <c r="IA97" t="inlineStr"/>
-      <c r="IB97" t="inlineStr"/>
-      <c r="IC97" t="inlineStr"/>
-      <c r="ID97" t="inlineStr"/>
-      <c r="IE97" t="inlineStr"/>
-      <c r="IF97" t="inlineStr"/>
-      <c r="IG97" t="inlineStr"/>
-      <c r="IH97" t="inlineStr"/>
-      <c r="II97" t="inlineStr"/>
-      <c r="IJ97" t="inlineStr"/>
-      <c r="IK97" t="inlineStr"/>
-      <c r="IL97" t="inlineStr"/>
-      <c r="IM97" t="inlineStr"/>
-      <c r="IN97" t="inlineStr"/>
-      <c r="IO97" t="inlineStr"/>
-      <c r="IP97" t="inlineStr"/>
-      <c r="IQ97" t="inlineStr"/>
-      <c r="IR97" t="inlineStr"/>
-      <c r="IS97" t="inlineStr"/>
-      <c r="IT97" t="inlineStr"/>
-      <c r="IU97" t="inlineStr"/>
-      <c r="IV97" t="inlineStr"/>
-      <c r="IW97" t="inlineStr"/>
-      <c r="IX97" t="inlineStr"/>
-      <c r="IY97" t="inlineStr"/>
-      <c r="IZ97" t="inlineStr"/>
-      <c r="JA97" t="inlineStr"/>
-      <c r="JB97" t="inlineStr"/>
-      <c r="JC97" t="inlineStr"/>
-      <c r="JD97" t="inlineStr"/>
-      <c r="JE97" t="inlineStr"/>
-      <c r="JF97" t="inlineStr"/>
-      <c r="JG97" t="inlineStr"/>
-      <c r="JH97" t="inlineStr"/>
-      <c r="JI97" t="inlineStr"/>
-      <c r="JJ97" t="inlineStr"/>
-      <c r="JK97" t="inlineStr"/>
-      <c r="JL97" t="inlineStr"/>
-      <c r="JM97" t="inlineStr"/>
-      <c r="JN97" t="inlineStr"/>
-      <c r="JO97" t="inlineStr"/>
-      <c r="JP97" t="inlineStr"/>
-      <c r="JQ97" t="inlineStr"/>
-      <c r="JR97" t="inlineStr"/>
-      <c r="JS97" t="inlineStr"/>
-      <c r="JT97" t="inlineStr"/>
-      <c r="JU97" t="inlineStr"/>
-      <c r="JV97" t="inlineStr"/>
-      <c r="JW97" t="inlineStr"/>
-      <c r="JX97" t="inlineStr"/>
-      <c r="JY97" t="inlineStr"/>
-      <c r="JZ97" t="inlineStr"/>
-      <c r="KA97" t="inlineStr"/>
-      <c r="KB97" t="inlineStr"/>
-      <c r="KC97" t="inlineStr"/>
-      <c r="KD97" t="inlineStr"/>
-      <c r="KE97" t="inlineStr"/>
-      <c r="KF97" t="inlineStr"/>
-      <c r="KG97" t="inlineStr"/>
-      <c r="KH97" t="inlineStr"/>
-      <c r="KI97" t="inlineStr"/>
-      <c r="KJ97" t="inlineStr"/>
-      <c r="KK97" t="inlineStr"/>
-      <c r="KL97" t="inlineStr"/>
-      <c r="KM97" t="inlineStr"/>
-      <c r="KN97" t="inlineStr"/>
-      <c r="KO97" t="inlineStr"/>
-      <c r="KP97" t="inlineStr"/>
-      <c r="KQ97" t="inlineStr"/>
-      <c r="KR97" t="inlineStr"/>
-      <c r="KS97" t="inlineStr"/>
-      <c r="KT97" t="inlineStr"/>
-      <c r="KU97" t="inlineStr"/>
-      <c r="KV97" t="inlineStr"/>
-      <c r="KW97" t="inlineStr"/>
-      <c r="KX97" t="inlineStr"/>
-      <c r="KY97" t="inlineStr"/>
-      <c r="KZ97" t="inlineStr"/>
-      <c r="LA97" t="inlineStr"/>
-      <c r="LB97" t="inlineStr"/>
-      <c r="LC97" t="inlineStr"/>
-      <c r="LD97" t="inlineStr"/>
-      <c r="LE97" t="inlineStr"/>
-      <c r="LF97" t="inlineStr"/>
-      <c r="LG97" t="inlineStr"/>
-      <c r="LH97" t="inlineStr"/>
-      <c r="LI97" t="inlineStr"/>
-      <c r="LJ97" t="inlineStr"/>
-      <c r="LK97" t="inlineStr"/>
-      <c r="LL97" t="inlineStr"/>
-      <c r="LM97" t="inlineStr"/>
-      <c r="LN97" t="inlineStr"/>
-      <c r="LO97" t="inlineStr"/>
-      <c r="LP97" t="inlineStr"/>
-      <c r="LQ97" t="inlineStr"/>
-      <c r="LR97" t="inlineStr"/>
-      <c r="LS97" t="inlineStr"/>
-      <c r="LT97" t="inlineStr"/>
-      <c r="LU97" t="inlineStr"/>
-      <c r="LV97" t="inlineStr"/>
-      <c r="LW97" t="inlineStr"/>
-      <c r="LX97" t="inlineStr"/>
-      <c r="LY97" t="inlineStr"/>
-      <c r="LZ97" t="inlineStr"/>
-      <c r="MA97" t="inlineStr"/>
-      <c r="MB97" t="inlineStr"/>
-      <c r="MC97" t="inlineStr"/>
-      <c r="MD97" t="inlineStr"/>
-      <c r="ME97" t="inlineStr"/>
-      <c r="MF97" t="inlineStr"/>
-      <c r="MG97" t="inlineStr"/>
-      <c r="MH97" t="inlineStr"/>
-      <c r="MI97" t="inlineStr"/>
-      <c r="MJ97" t="inlineStr"/>
-      <c r="MK97" t="inlineStr"/>
-      <c r="ML97" t="inlineStr"/>
-      <c r="MM97" t="inlineStr"/>
-      <c r="MN97" t="inlineStr"/>
-      <c r="MO97" t="inlineStr"/>
-      <c r="MP97" t="inlineStr"/>
-      <c r="MQ97" t="inlineStr"/>
-      <c r="MR97" t="inlineStr"/>
-      <c r="MS97" t="inlineStr"/>
-      <c r="MT97" t="inlineStr"/>
-      <c r="MU97" t="inlineStr"/>
-      <c r="MV97" t="inlineStr"/>
-      <c r="MW97" t="inlineStr"/>
-      <c r="MX97" t="inlineStr"/>
-      <c r="MY97" t="inlineStr"/>
-      <c r="MZ97" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>